<commit_message>
Issue #5: publish Final3 Copilot and PAD acceptance evidence
</commit_message>
<xml_diff>
--- a/catalog/evidence/copilot-excel-t10-v6.xlsx
+++ b/catalog/evidence/copilot-excel-t10-v6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuuki\ai-prompts\catalog\evidence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F199B334-3355-4CE7-B8A2-991265D52D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4EE31F69-F70F-462D-86BB-78EE0FFB9A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5A79F3E5-511E-4837-A908-59DE5CC6B197}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{80B571CB-BD79-4E4F-BB49-A1213FF96737}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -424,7 +424,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0F301FE-BB66-4277-945A-3AC8EF27A8DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED9854C3-24C4-442B-8393-F05D86DC88CF}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <sheetData>

</xml_diff>